<commit_message>
import morphotypes, vernacular names in custom taxonomy
</commit_message>
<xml_diff>
--- a/app_kit/tests/TESTS_ROOT/xlsx_for_testing/TaxonProfiles/invalid/Taxon profiles.xlsx
+++ b/app_kit/tests/TESTS_ROOT/xlsx_for_testing/TaxonProfiles/invalid/Taxon profiles.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
   <si>
     <t xml:space="preserve">Scientific Names</t>
   </si>
@@ -30,6 +30,9 @@
   </si>
   <si>
     <t xml:space="preserve">Morphotype (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object class (optional)</t>
   </si>
   <si>
     <t xml:space="preserve">short_profile</t>
@@ -427,37 +430,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -530,18 +533,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMR27"/>
+  <dimension ref="A1:AMS27"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="38.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="47.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="47.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="38.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="8" style="2" width="31.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="16" style="2" width="17.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="2" width="21.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="47.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="47.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="38.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="9" style="2" width="31.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="22.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="17" style="2" width="17.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="2" width="21.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -555,41 +558,41 @@
       <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="G1" s="4"/>
       <c r="H1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="4"/>
+      <c r="J1" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="K1" s="4"/>
-      <c r="L1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>7</v>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S1" s="5" t="s">
         <v>9</v>
@@ -597,7 +600,9 @@
       <c r="T1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="U1" s="5"/>
+      <c r="U1" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="V1" s="5"/>
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
@@ -1609,21 +1614,20 @@
       <c r="AMP1" s="5"/>
       <c r="AMQ1" s="5"/>
       <c r="AMR1" s="5"/>
+      <c r="AMS1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4" t="s">
-        <v>11</v>
-      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
       <c r="G2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>13</v>
@@ -1635,23 +1639,25 @@
         <v>15</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5" t="s">
         <v>16</v>
       </c>
+      <c r="M2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="5"/>
       <c r="O2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5" t="s">
-        <v>16</v>
-      </c>
+      <c r="P2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="S2" s="5"/>
+        <v>17</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="T2" s="5"/>
       <c r="U2" s="5"/>
       <c r="V2" s="5"/>
@@ -2665,27 +2671,28 @@
       <c r="AMP2" s="5"/>
       <c r="AMQ2" s="5"/>
       <c r="AMR2" s="5"/>
+      <c r="AMS2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
-      <c r="E3" s="4"/>
+      <c r="E3" s="3"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="4" t="s">
-        <v>19</v>
-      </c>
+      <c r="J3" s="4"/>
       <c r="K3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3" s="5"/>
+        <v>20</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
@@ -3705,21 +3712,19 @@
       <c r="AMP3" s="5"/>
       <c r="AMQ3" s="5"/>
       <c r="AMR3" s="5"/>
+      <c r="AMS3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>24</v>
       </c>
       <c r="I4" s="6" t="s">
@@ -3734,248 +3739,252 @@
       <c r="L4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N4" s="8"/>
+      <c r="N4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="191.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="9"/>
+        <v>22</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>32</v>
+      </c>
       <c r="H5" s="9"/>
-      <c r="I5" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
-      <c r="M5" s="2" t="s">
-        <v>33</v>
+      <c r="M5" s="9"/>
+      <c r="N5" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="6"/>
+        <v>22</v>
+      </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="6"/>
+        <v>22</v>
+      </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
       <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F16" s="6"/>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
       <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="112.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
-      <c r="F18" s="11"/>
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
       <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
       <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
       <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F21" s="12"/>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F22" s="12"/>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
       <c r="K22" s="12"/>
       <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F23" s="12"/>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
       <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F24" s="12"/>
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
       <c r="K24" s="12"/>
       <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F25" s="12"/>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
       <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F26" s="12"/>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
       <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F27" s="12"/>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="F5:H5"/>
+  <mergeCells count="2">
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:M5"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
@@ -4007,57 +4016,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>